<commit_message>
example 1 preliminary draft
</commit_message>
<xml_diff>
--- a/data/example_01.xlsx
+++ b/data/example_01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdagcc-my.sharepoint.com/personal/nora_bello_usda_gov/Documents/Documents/Consulting&amp;Collaborations/Stroup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpiaskowski\Documents\git\glmm-guide\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DF8D072C-3004-4628-A5CA-855CCD8FE1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261C992A-D4E1-4807-93A5-E265904FBED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26880" yWindow="1530" windowWidth="21600" windowHeight="11235" xr2:uid="{1A013764-9008-4C39-AFE0-5E18C046064B}"/>
+    <workbookView xWindow="18050" yWindow="810" windowWidth="19400" windowHeight="17500" xr2:uid="{1A013764-9008-4C39-AFE0-5E18C046064B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -417,9 +417,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CDCF6D-B9F0-4ACD-818A-A397170CD7BC}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -430,7 +430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -441,7 +441,7 @@
         <v>24.739000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -452,7 +452,7 @@
         <v>22.719000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -463,7 +463,7 @@
         <v>27.247</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -474,7 +474,7 @@
         <v>28.45</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -485,7 +485,7 @@
         <v>30.202000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -496,7 +496,7 @@
         <v>30.422000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -507,7 +507,7 @@
         <v>27.920999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2</v>
       </c>
@@ -518,7 +518,7 @@
         <v>29.419</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
@@ -529,7 +529,7 @@
         <v>27.024999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2</v>
       </c>
@@ -540,7 +540,7 @@
         <v>30.466999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2</v>
       </c>
@@ -551,7 +551,7 @@
         <v>23.334</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2</v>
       </c>
@@ -562,7 +562,7 @@
         <v>23.298999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>3</v>
       </c>
@@ -573,7 +573,7 @@
         <v>24.064</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>3</v>
       </c>
@@ -584,7 +584,7 @@
         <v>22.945</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>3</v>
       </c>
@@ -595,7 +595,7 @@
         <v>26.169</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>3</v>
       </c>
@@ -606,7 +606,7 @@
         <v>30.414000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>3</v>
       </c>
@@ -617,7 +617,7 @@
         <v>28.661000000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>3</v>
       </c>
@@ -628,7 +628,7 @@
         <v>29.571000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>4</v>
       </c>
@@ -639,7 +639,7 @@
         <v>25.102</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>4</v>
       </c>
@@ -650,7 +650,7 @@
         <v>28.341999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>4</v>
       </c>
@@ -661,7 +661,7 @@
         <v>29.337</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>4</v>
       </c>
@@ -672,7 +672,7 @@
         <v>23.713999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>4</v>
       </c>
@@ -683,7 +683,7 @@
         <v>33.414000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>4</v>
       </c>
@@ -694,7 +694,7 @@
         <v>26.562999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>5</v>
       </c>
@@ -705,7 +705,7 @@
         <v>22.352</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>5</v>
       </c>
@@ -716,7 +716,7 @@
         <v>30.347999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>5</v>
       </c>
@@ -727,7 +727,7 @@
         <v>23.797999999999998</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>5</v>
       </c>
@@ -738,7 +738,7 @@
         <v>29.196999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>5</v>
       </c>
@@ -749,7 +749,7 @@
         <v>30.625</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>5</v>
       </c>

</xml_diff>